<commit_message>
updated according to requirements
</commit_message>
<xml_diff>
--- a/April submission/Week-2/project/back/template/quotation_template.xlsx
+++ b/April submission/Week-2/project/back/template/quotation_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\College\8th Sem\Shivvilon Solutions\April submission\Week-2\project\back\src\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\College\8th Sem\Shivvilon Solutions\April submission\Week-2\project\back\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F5EEE2-7655-4DC5-957F-CE79B4A31E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF241407-BE3D-4481-9ECA-818EA52B8080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="11092017" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="23">
   <si>
     <t>ADD:-</t>
   </si>
@@ -65,9 +65,6 @@
     <t>DELI TIME:-</t>
   </si>
   <si>
-    <t>MO</t>
-  </si>
-  <si>
     <t>PIC</t>
   </si>
   <si>
@@ -80,30 +77,35 @@
     <t>SHREE:-</t>
   </si>
   <si>
-    <t>MO:-9925018479</t>
-  </si>
-  <si>
     <t xml:space="preserve">RATE B:- </t>
   </si>
   <si>
-    <t xml:space="preserve">કટિંગ કરેલ માલ પાછો રાખવા માં નહિ આવે
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD:- </t>
+  </si>
+  <si>
+    <t>MO:- 9879264139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BENDING:- </t>
+  </si>
+  <si>
+    <t>કટીંગમાં 0.5 MM નું વેરિયેશન રહેશે</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
 </t>
   </si>
   <si>
-    <t xml:space="preserve">માપ ચેક કરી ને રજા લેવી
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADD:- </t>
-  </si>
-  <si>
-    <t>MO:- 9879264139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BENDING:- </t>
+    <t>TOTAL PIECE</t>
+  </si>
+  <si>
+    <t>MOBILE NO:-</t>
+  </si>
+  <si>
+    <t>RATE W:-</t>
   </si>
 </sst>
 </file>
@@ -160,7 +162,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -503,48 +505,82 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -555,7 +591,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -646,23 +682,53 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -671,16 +737,25 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1004,30 +1079,27 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="21"/>
-      <c r="C1" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="49"/>
-      <c r="E1" s="50"/>
+      <c r="C1" s="63" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="63"/>
+      <c r="E1" s="64"/>
       <c r="F1" s="36" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="48"/>
+      <c r="C2" s="58"/>
       <c r="D2" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="20">
-        <f ca="1">NOW()</f>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="12">
@@ -1048,7 +1120,7 @@
       <c r="D4" s="27"/>
       <c r="E4" s="25"/>
       <c r="F4" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
@@ -1059,7 +1131,7 @@
       <c r="D5" s="26"/>
       <c r="E5" s="25"/>
       <c r="F5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
@@ -1079,12 +1151,12 @@
         <v>5</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D7" s="26"/>
       <c r="E7" s="25"/>
       <c r="F7" s="40" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1095,55 +1167,60 @@
       <c r="D8" s="30"/>
       <c r="E8" s="39"/>
       <c r="F8" s="38" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="45"/>
-    </row>
-    <row r="10" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="48"/>
+      <c r="B9" s="54">
+        <v>7</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="60"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="55">
+        <v>9925018479</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="48"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="42">
+        <v>9825018420</v>
+      </c>
     </row>
     <row r="11" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="21"/>
-      <c r="C11" s="49" t="str">
+      <c r="B11" s="52"/>
+      <c r="C11" s="63" t="str">
         <f>C1</f>
         <v>SHREE:-</v>
       </c>
-      <c r="D11" s="49"/>
-      <c r="E11" s="50"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="64"/>
       <c r="F11" s="36" t="str">
         <f t="shared" ref="F11:F17" si="0">F1</f>
         <v>DELI TIME:-</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="48"/>
+      <c r="C12" s="58"/>
       <c r="D12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="20">
-        <f t="shared" ca="1" si="0"/>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F12" s="20"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="12">
@@ -1213,55 +1290,60 @@
       <c r="D18" s="30"/>
       <c r="E18" s="39"/>
       <c r="F18" s="38" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="45"/>
-    </row>
-    <row r="20" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="48"/>
+      <c r="B19" s="54">
+        <v>7</v>
+      </c>
+      <c r="C19" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="60"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="55">
+        <v>9925018479</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="48"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="42">
+        <v>9825018420</v>
+      </c>
     </row>
     <row r="21" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="21"/>
-      <c r="C21" s="49" t="str">
+      <c r="B21" s="52"/>
+      <c r="C21" s="63" t="str">
         <f>C1</f>
         <v>SHREE:-</v>
       </c>
-      <c r="D21" s="49"/>
-      <c r="E21" s="50"/>
+      <c r="D21" s="63"/>
+      <c r="E21" s="64"/>
       <c r="F21" s="36" t="str">
         <f t="shared" ref="F21:F27" si="1">F1</f>
         <v>DELI TIME:-</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="48"/>
+      <c r="C22" s="58"/>
       <c r="D22" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="20">
-        <f t="shared" ca="1" si="1"/>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F22" s="20"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="12">
@@ -1331,44 +1413,49 @@
       <c r="D28" s="30"/>
       <c r="E28" s="39"/>
       <c r="F28" s="38" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="45"/>
-    </row>
-    <row r="30" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="48"/>
+      <c r="B29" s="54">
+        <v>7</v>
+      </c>
+      <c r="C29" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="60"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="55">
+        <v>9925018479</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="71"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="42">
+        <v>9825018420</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
+  <mergeCells count="9">
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B9:F9"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B20:F20"/>
   </mergeCells>
   <pageMargins left="2.0099999999999998" right="2.0499999999999998" top="0.16" bottom="5.88" header="0.16" footer="0.3"/>
-  <pageSetup paperSize="9" scale="89" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="89" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1386,30 +1473,27 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="22"/>
-      <c r="C1" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="52"/>
+      <c r="C1" s="66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="66"/>
+      <c r="E1" s="67"/>
       <c r="F1" s="31" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="54"/>
+      <c r="C2" s="70"/>
       <c r="D2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="5">
-        <f ca="1">NOW()</f>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="6">
@@ -1419,7 +1503,7 @@
       <c r="D3" s="25"/>
       <c r="E3" s="25"/>
       <c r="F3" s="32" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
@@ -1429,7 +1513,9 @@
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="25"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="6">
@@ -1450,7 +1536,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="25"/>
       <c r="F6" s="33" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -1481,7 +1567,7 @@
       <c r="D9" s="26"/>
       <c r="E9" s="25"/>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
@@ -1515,62 +1601,58 @@
       <c r="E12" s="25"/>
       <c r="F12" s="40"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="19">
         <v>11</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="25"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="39"/>
       <c r="F13" s="41"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="26">
+    <row r="14" spans="2:6" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="51">
         <v>12</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="42"/>
-    </row>
-    <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="4">
-        <v>13</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4">
-        <f>SUM(D3:D14)</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="40"/>
+      <c r="C14" s="57" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="65"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="46"/>
+    </row>
+    <row r="15" spans="2:6" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="43"/>
+      <c r="C15" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="44"/>
     </row>
     <row r="16" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="22"/>
-      <c r="C16" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="51"/>
-      <c r="E16" s="52"/>
+      <c r="C16" s="68" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="66"/>
+      <c r="E16" s="67"/>
       <c r="F16" s="31" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="54"/>
+      <c r="C17" s="70"/>
       <c r="D17" s="3" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F17" s="5">
-        <f ca="1">NOW()</f>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18" s="6">
@@ -1580,7 +1662,7 @@
       <c r="D18" s="25"/>
       <c r="E18" s="25"/>
       <c r="F18" s="32" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.3">
@@ -1590,7 +1672,9 @@
       <c r="C19" s="26"/>
       <c r="D19" s="27"/>
       <c r="E19" s="25"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B20" s="6">
@@ -1611,7 +1695,7 @@
       <c r="D21" s="26"/>
       <c r="E21" s="25"/>
       <c r="F21" s="33" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
@@ -1643,7 +1727,7 @@
       <c r="D24" s="26"/>
       <c r="E24" s="25"/>
       <c r="F24" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.3">
@@ -1677,46 +1761,47 @@
       <c r="E27" s="25"/>
       <c r="F27" s="40"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="19">
         <v>11</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="25"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="39"/>
       <c r="F28" s="41"/>
     </row>
-    <row r="29" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="26">
+    <row r="29" spans="2:7" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="51">
         <v>12</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="42"/>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B30" s="4">
-        <v>13</v>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4">
-        <f>SUM(D18:D29)</f>
-        <v>0</v>
-      </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="40"/>
+      <c r="C29" s="57" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="65"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="46"/>
+    </row>
+    <row r="30" spans="2:7" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="43"/>
+      <c r="C30" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="44"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="D31" s="9"/>
       <c r="E31" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="1.78" right="2.2999999999999998" top="0.18" bottom="5.93" header="0.16" footer="0.3"/>
   <pageSetup paperSize="9" scale="89" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -1738,30 +1823,27 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="21"/>
-      <c r="C1" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="51"/>
-      <c r="E1" s="52"/>
+      <c r="C1" s="66" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="66"/>
+      <c r="E1" s="67"/>
       <c r="F1" s="31" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="48"/>
+      <c r="C2" s="58"/>
       <c r="D2" s="13" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="14">
-        <f ca="1">NOW()</f>
-        <v>46161.715168055554</v>
-      </c>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="12">
@@ -1781,7 +1863,9 @@
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="25"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="6">
@@ -1813,7 +1897,7 @@
       <c r="D7" s="26"/>
       <c r="E7" s="25"/>
       <c r="F7" s="23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
@@ -1833,7 +1917,7 @@
       <c r="D9" s="26"/>
       <c r="E9" s="25"/>
       <c r="F9" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2003,7 +2087,7 @@
       <c r="F27" s="40"/>
     </row>
     <row r="28" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="41">
+      <c r="B28" s="16">
         <v>26</v>
       </c>
       <c r="C28" s="16"/>
@@ -2012,22 +2096,24 @@
       <c r="F28" s="41"/>
     </row>
     <row r="29" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="45"/>
+      <c r="B29" s="45">
+        <v>27</v>
+      </c>
+      <c r="C29" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="60"/>
+      <c r="E29" s="61"/>
+      <c r="F29" s="46"/>
     </row>
     <row r="30" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="46" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="48"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="49"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B31" s="15"/>
@@ -2036,11 +2122,10 @@
       <c r="B32" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="C1:E1"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="C29:E29"/>
   </mergeCells>
   <pageMargins left="2.12" right="1.88" top="0.2" bottom="0.8" header="0.16" footer="5.88"/>
   <pageSetup paperSize="9" scale="89" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>